<commit_message>
feat: persist email credentials in browser localStorage + env vars so users never re-type App Password on server restarts
</commit_message>
<xml_diff>
--- a/sample_data/Certification - Participation stats.preprocessed (2)_1785172035.xlsx
+++ b/sample_data/Certification - Participation stats.preprocessed (2)_1785172035.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Amal\Downloads\cert_automation\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F3DC4A9-6BF0-4F68-B9C3-5C85A2C283F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FF3B924-16D5-4BB4-8ADD-A8D651D81E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4546,9 +4546,6 @@
     <t>Institution</t>
   </si>
   <si>
-    <t>amal.tom@btech.christuniversity.in</t>
-  </si>
-  <si>
     <t>aimy.tom@btech.christuniversity.in</t>
   </si>
   <si>
@@ -4562,6 +4559,9 @@
   </si>
   <si>
     <t>Ms. Salomi Gopinath</t>
+  </si>
+  <si>
+    <t>amaltomajithp@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -4889,11 +4889,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4903,6 +4898,11 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -5135,7 +5135,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="54" t="s">
         <v>1507</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -5164,11 +5164,11 @@
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="59" t="s">
-        <v>1511</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>1508</v>
+      <c r="B2" s="56" t="s">
+        <v>1510</v>
+      </c>
+      <c r="C2" s="55" t="s">
+        <v>1513</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>8</v>
@@ -5190,11 +5190,11 @@
       <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="59" t="s">
-        <v>1511</v>
-      </c>
-      <c r="C3" s="58" t="s">
-        <v>1508</v>
+      <c r="B3" s="56" t="s">
+        <v>1510</v>
+      </c>
+      <c r="C3" s="55" t="s">
+        <v>1513</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>13</v>
@@ -5216,11 +5216,11 @@
       <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="59" t="s">
-        <v>1511</v>
-      </c>
-      <c r="C4" s="58" t="s">
-        <v>1508</v>
+      <c r="B4" s="56" t="s">
+        <v>1510</v>
+      </c>
+      <c r="C4" s="55" t="s">
+        <v>1513</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>14</v>
@@ -5242,11 +5242,11 @@
       <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="59" t="s">
-        <v>1511</v>
-      </c>
-      <c r="C5" s="58" t="s">
-        <v>1508</v>
+      <c r="B5" s="56" t="s">
+        <v>1510</v>
+      </c>
+      <c r="C5" s="55" t="s">
+        <v>1513</v>
       </c>
       <c r="D5" s="6" t="s">
         <v>15</v>
@@ -5268,11 +5268,11 @@
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="59" t="s">
-        <v>1511</v>
-      </c>
-      <c r="C6" s="58" t="s">
-        <v>1508</v>
+      <c r="B6" s="56" t="s">
+        <v>1510</v>
+      </c>
+      <c r="C6" s="55" t="s">
+        <v>1513</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>17</v>
@@ -5294,11 +5294,11 @@
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="59" t="s">
-        <v>1511</v>
-      </c>
-      <c r="C7" s="58" t="s">
-        <v>1508</v>
+      <c r="B7" s="56" t="s">
+        <v>1510</v>
+      </c>
+      <c r="C7" s="55" t="s">
+        <v>1513</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>18</v>
@@ -5320,11 +5320,11 @@
       <c r="A8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="59" t="s">
-        <v>1511</v>
-      </c>
-      <c r="C8" s="58" t="s">
-        <v>1508</v>
+      <c r="B8" s="56" t="s">
+        <v>1510</v>
+      </c>
+      <c r="C8" s="55" t="s">
+        <v>1513</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>19</v>
@@ -5346,11 +5346,11 @@
       <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="59" t="s">
-        <v>1511</v>
-      </c>
-      <c r="C9" s="58" t="s">
-        <v>1508</v>
+      <c r="B9" s="56" t="s">
+        <v>1510</v>
+      </c>
+      <c r="C9" s="55" t="s">
+        <v>1513</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>20</v>
@@ -5372,11 +5372,11 @@
       <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="59" t="s">
-        <v>1511</v>
-      </c>
-      <c r="C10" s="58" t="s">
-        <v>1508</v>
+      <c r="B10" s="56" t="s">
+        <v>1510</v>
+      </c>
+      <c r="C10" s="55" t="s">
+        <v>1513</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>21</v>
@@ -5398,11 +5398,11 @@
       <c r="A11" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="59" t="s">
-        <v>1511</v>
-      </c>
-      <c r="C11" s="58" t="s">
-        <v>1508</v>
+      <c r="B11" s="56" t="s">
+        <v>1510</v>
+      </c>
+      <c r="C11" s="55" t="s">
+        <v>1513</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>22</v>
@@ -5424,11 +5424,11 @@
       <c r="A12" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="59" t="s">
-        <v>1510</v>
-      </c>
-      <c r="C12" s="58" t="s">
+      <c r="B12" s="56" t="s">
         <v>1509</v>
+      </c>
+      <c r="C12" s="55" t="s">
+        <v>1508</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>24</v>
@@ -5446,11 +5446,11 @@
       <c r="A13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="59" t="s">
-        <v>1510</v>
-      </c>
-      <c r="C13" s="58" t="s">
+      <c r="B13" s="56" t="s">
         <v>1509</v>
+      </c>
+      <c r="C13" s="55" t="s">
+        <v>1508</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>25</v>
@@ -5468,11 +5468,11 @@
       <c r="A14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="59" t="s">
-        <v>1510</v>
-      </c>
-      <c r="C14" s="58" t="s">
+      <c r="B14" s="56" t="s">
         <v>1509</v>
+      </c>
+      <c r="C14" s="55" t="s">
+        <v>1508</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>26</v>
@@ -5490,11 +5490,11 @@
       <c r="A15" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="59" t="s">
-        <v>1510</v>
-      </c>
-      <c r="C15" s="58" t="s">
+      <c r="B15" s="56" t="s">
         <v>1509</v>
+      </c>
+      <c r="C15" s="55" t="s">
+        <v>1508</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>27</v>
@@ -5512,11 +5512,11 @@
       <c r="A16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="59" t="s">
-        <v>1510</v>
-      </c>
-      <c r="C16" s="58" t="s">
+      <c r="B16" s="56" t="s">
         <v>1509</v>
+      </c>
+      <c r="C16" s="55" t="s">
+        <v>1508</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>28</v>
@@ -5534,11 +5534,11 @@
       <c r="A17" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="59" t="s">
-        <v>1510</v>
-      </c>
-      <c r="C17" s="58" t="s">
+      <c r="B17" s="56" t="s">
         <v>1509</v>
+      </c>
+      <c r="C17" s="55" t="s">
+        <v>1508</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>29</v>
@@ -5556,11 +5556,11 @@
       <c r="A18" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="59" t="s">
-        <v>1510</v>
-      </c>
-      <c r="C18" s="58" t="s">
+      <c r="B18" s="56" t="s">
         <v>1509</v>
+      </c>
+      <c r="C18" s="55" t="s">
+        <v>1508</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>30</v>
@@ -5578,11 +5578,11 @@
       <c r="A19" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="59" t="s">
-        <v>1510</v>
-      </c>
-      <c r="C19" s="58" t="s">
+      <c r="B19" s="56" t="s">
         <v>1509</v>
+      </c>
+      <c r="C19" s="55" t="s">
+        <v>1508</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>31</v>
@@ -5600,11 +5600,11 @@
       <c r="A20" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="60" t="s">
-        <v>1513</v>
-      </c>
-      <c r="C20" s="61" t="s">
+      <c r="B20" s="57" t="s">
         <v>1512</v>
+      </c>
+      <c r="C20" s="58" t="s">
+        <v>1511</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>34</v>
@@ -5635,11 +5635,11 @@
       <c r="A21" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="60" t="s">
-        <v>1513</v>
-      </c>
-      <c r="C21" s="61" t="s">
+      <c r="B21" s="57" t="s">
         <v>1512</v>
+      </c>
+      <c r="C21" s="58" t="s">
+        <v>1511</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>35</v>
@@ -5661,11 +5661,11 @@
       <c r="A22" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B22" s="60" t="s">
-        <v>1513</v>
-      </c>
-      <c r="C22" s="61" t="s">
+      <c r="B22" s="57" t="s">
         <v>1512</v>
+      </c>
+      <c r="C22" s="58" t="s">
+        <v>1511</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>37</v>
@@ -5687,11 +5687,11 @@
       <c r="A23" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B23" s="60" t="s">
-        <v>1513</v>
-      </c>
-      <c r="C23" s="61" t="s">
+      <c r="B23" s="57" t="s">
         <v>1512</v>
+      </c>
+      <c r="C23" s="58" t="s">
+        <v>1511</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>38</v>
@@ -5713,11 +5713,11 @@
       <c r="A24" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="60" t="s">
-        <v>1513</v>
-      </c>
-      <c r="C24" s="61" t="s">
+      <c r="B24" s="57" t="s">
         <v>1512</v>
+      </c>
+      <c r="C24" s="58" t="s">
+        <v>1511</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>39</v>
@@ -5739,11 +5739,11 @@
       <c r="A25" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B25" s="60" t="s">
-        <v>1513</v>
-      </c>
-      <c r="C25" s="61" t="s">
+      <c r="B25" s="57" t="s">
         <v>1512</v>
+      </c>
+      <c r="C25" s="58" t="s">
+        <v>1511</v>
       </c>
       <c r="D25" s="6" t="s">
         <v>40</v>
@@ -5768,7 +5768,7 @@
       <c r="B26" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C26" s="58"/>
+      <c r="C26" s="55"/>
       <c r="D26" s="6" t="s">
         <v>43</v>
       </c>
@@ -5792,7 +5792,7 @@
       <c r="B27" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C27" s="58"/>
+      <c r="C27" s="55"/>
       <c r="D27" s="6" t="s">
         <v>46</v>
       </c>
@@ -5816,7 +5816,7 @@
       <c r="B28" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C28" s="58"/>
+      <c r="C28" s="55"/>
       <c r="D28" s="6" t="s">
         <v>47</v>
       </c>
@@ -5840,7 +5840,7 @@
       <c r="B29" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C29" s="58"/>
+      <c r="C29" s="55"/>
       <c r="D29" s="6" t="s">
         <v>48</v>
       </c>
@@ -5864,7 +5864,7 @@
       <c r="B30" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="58"/>
+      <c r="C30" s="55"/>
       <c r="D30" s="6" t="s">
         <v>49</v>
       </c>
@@ -5888,7 +5888,7 @@
       <c r="B31" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C31" s="58"/>
+      <c r="C31" s="55"/>
       <c r="D31" s="6" t="s">
         <v>50</v>
       </c>
@@ -5912,7 +5912,7 @@
       <c r="B32" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C32" s="58"/>
+      <c r="C32" s="55"/>
       <c r="D32" s="6" t="s">
         <v>51</v>
       </c>
@@ -5936,7 +5936,7 @@
       <c r="B33" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C33" s="58"/>
+      <c r="C33" s="55"/>
       <c r="D33" s="6" t="s">
         <v>54</v>
       </c>
@@ -5960,7 +5960,7 @@
       <c r="B34" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C34" s="58"/>
+      <c r="C34" s="55"/>
       <c r="D34" s="6" t="s">
         <v>56</v>
       </c>
@@ -5984,7 +5984,7 @@
       <c r="B35" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C35" s="58"/>
+      <c r="C35" s="55"/>
       <c r="D35" s="6" t="s">
         <v>57</v>
       </c>
@@ -6008,7 +6008,7 @@
       <c r="B36" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C36" s="58"/>
+      <c r="C36" s="55"/>
       <c r="D36" s="6" t="s">
         <v>58</v>
       </c>
@@ -6032,7 +6032,7 @@
       <c r="B37" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C37" s="58"/>
+      <c r="C37" s="55"/>
       <c r="D37" s="6" t="s">
         <v>59</v>
       </c>
@@ -6056,7 +6056,7 @@
       <c r="B38" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C38" s="58"/>
+      <c r="C38" s="55"/>
       <c r="D38" s="6" t="s">
         <v>60</v>
       </c>
@@ -6080,7 +6080,7 @@
       <c r="B39" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C39" s="58"/>
+      <c r="C39" s="55"/>
       <c r="D39" s="6" t="s">
         <v>63</v>
       </c>
@@ -6104,7 +6104,7 @@
       <c r="B40" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C40" s="58"/>
+      <c r="C40" s="55"/>
       <c r="D40" s="6" t="s">
         <v>65</v>
       </c>
@@ -7294,7 +7294,7 @@
       <c r="F90" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G90" s="56" t="s">
+      <c r="G90" s="61" t="s">
         <v>134</v>
       </c>
       <c r="H90" s="7" t="s">
@@ -7316,7 +7316,7 @@
       <c r="F91" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G91" s="55"/>
+      <c r="G91" s="60"/>
       <c r="H91" s="7" t="s">
         <v>12</v>
       </c>
@@ -7336,7 +7336,7 @@
       <c r="F92" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G92" s="55"/>
+      <c r="G92" s="60"/>
       <c r="H92" s="7" t="s">
         <v>12</v>
       </c>
@@ -7356,7 +7356,7 @@
       <c r="F93" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G93" s="55"/>
+      <c r="G93" s="60"/>
       <c r="H93" s="7" t="s">
         <v>12</v>
       </c>
@@ -7376,7 +7376,7 @@
       <c r="F94" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G94" s="55"/>
+      <c r="G94" s="60"/>
       <c r="H94" s="7" t="s">
         <v>12</v>
       </c>
@@ -7396,7 +7396,7 @@
       <c r="F95" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G95" s="55"/>
+      <c r="G95" s="60"/>
       <c r="H95" s="7" t="s">
         <v>12</v>
       </c>
@@ -7416,7 +7416,7 @@
       <c r="F96" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G96" s="55"/>
+      <c r="G96" s="60"/>
       <c r="H96" s="7" t="s">
         <v>12</v>
       </c>
@@ -7436,7 +7436,7 @@
       <c r="F97" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G97" s="55"/>
+      <c r="G97" s="60"/>
       <c r="H97" s="7" t="s">
         <v>12</v>
       </c>
@@ -7456,7 +7456,7 @@
       <c r="F98" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G98" s="55"/>
+      <c r="G98" s="60"/>
       <c r="H98" s="7" t="s">
         <v>12</v>
       </c>
@@ -12634,7 +12634,7 @@
       <c r="F316" s="15" t="s">
         <v>352</v>
       </c>
-      <c r="G316" s="54" t="s">
+      <c r="G316" s="59" t="s">
         <v>448</v>
       </c>
       <c r="H316" s="7" t="s">
@@ -12658,7 +12658,7 @@
       <c r="F317" s="15" t="s">
         <v>352</v>
       </c>
-      <c r="G317" s="55"/>
+      <c r="G317" s="60"/>
       <c r="H317" s="7" t="s">
         <v>420</v>
       </c>
@@ -12680,7 +12680,7 @@
       <c r="F318" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="G318" s="54" t="s">
+      <c r="G318" s="59" t="s">
         <v>451</v>
       </c>
       <c r="H318" s="7" t="s">
@@ -12704,7 +12704,7 @@
       <c r="F319" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="G319" s="55"/>
+      <c r="G319" s="60"/>
       <c r="H319" s="7" t="s">
         <v>420</v>
       </c>
@@ -13086,7 +13086,7 @@
       <c r="F335" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G335" s="54" t="s">
+      <c r="G335" s="59" t="s">
         <v>472</v>
       </c>
       <c r="H335" s="7" t="s">
@@ -13110,7 +13110,7 @@
       <c r="F336" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G336" s="55"/>
+      <c r="G336" s="60"/>
       <c r="H336" s="7" t="s">
         <v>420</v>
       </c>
@@ -13132,7 +13132,7 @@
       <c r="F337" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G337" s="55"/>
+      <c r="G337" s="60"/>
       <c r="H337" s="7" t="s">
         <v>420</v>
       </c>
@@ -13154,7 +13154,7 @@
       <c r="F338" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="G338" s="54" t="s">
+      <c r="G338" s="59" t="s">
         <v>476</v>
       </c>
       <c r="H338" s="7" t="s">
@@ -13178,7 +13178,7 @@
       <c r="F339" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="G339" s="55"/>
+      <c r="G339" s="60"/>
       <c r="H339" s="7" t="s">
         <v>420</v>
       </c>
@@ -13200,7 +13200,7 @@
       <c r="F340" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="G340" s="55"/>
+      <c r="G340" s="60"/>
       <c r="H340" s="7" t="s">
         <v>420</v>
       </c>
@@ -13222,7 +13222,7 @@
       <c r="F341" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G341" s="54" t="s">
+      <c r="G341" s="59" t="s">
         <v>480</v>
       </c>
       <c r="H341" s="7" t="s">
@@ -13246,7 +13246,7 @@
       <c r="F342" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G342" s="55"/>
+      <c r="G342" s="60"/>
       <c r="H342" s="7" t="s">
         <v>420</v>
       </c>
@@ -13268,7 +13268,7 @@
       <c r="F343" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G343" s="55"/>
+      <c r="G343" s="60"/>
       <c r="H343" s="7" t="s">
         <v>420</v>
       </c>
@@ -13290,7 +13290,7 @@
       <c r="F344" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G344" s="55"/>
+      <c r="G344" s="60"/>
       <c r="H344" s="7" t="s">
         <v>420</v>
       </c>
@@ -13312,7 +13312,7 @@
       <c r="F345" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G345" s="55"/>
+      <c r="G345" s="60"/>
       <c r="H345" s="7" t="s">
         <v>420</v>
       </c>
@@ -13334,7 +13334,7 @@
       <c r="F346" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G346" s="54" t="s">
+      <c r="G346" s="59" t="s">
         <v>486</v>
       </c>
       <c r="H346" s="7" t="s">
@@ -13358,7 +13358,7 @@
       <c r="F347" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G347" s="55"/>
+      <c r="G347" s="60"/>
       <c r="H347" s="7" t="s">
         <v>420</v>
       </c>
@@ -13380,7 +13380,7 @@
       <c r="F348" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G348" s="55"/>
+      <c r="G348" s="60"/>
       <c r="H348" s="7" t="s">
         <v>420</v>
       </c>
@@ -13402,7 +13402,7 @@
       <c r="F349" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G349" s="55"/>
+      <c r="G349" s="60"/>
       <c r="H349" s="7" t="s">
         <v>420</v>
       </c>
@@ -13424,7 +13424,7 @@
       <c r="F350" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G350" s="54" t="s">
+      <c r="G350" s="59" t="s">
         <v>490</v>
       </c>
       <c r="H350" s="7" t="s">
@@ -13448,7 +13448,7 @@
       <c r="F351" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G351" s="55"/>
+      <c r="G351" s="60"/>
       <c r="H351" s="7" t="s">
         <v>420</v>
       </c>
@@ -13470,7 +13470,7 @@
       <c r="F352" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G352" s="55"/>
+      <c r="G352" s="60"/>
       <c r="H352" s="7" t="s">
         <v>420</v>
       </c>
@@ -13492,7 +13492,7 @@
       <c r="F353" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G353" s="55"/>
+      <c r="G353" s="60"/>
       <c r="H353" s="7" t="s">
         <v>420</v>
       </c>
@@ -13512,7 +13512,7 @@
       <c r="F354" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G354" s="54" t="s">
+      <c r="G354" s="59" t="s">
         <v>495</v>
       </c>
       <c r="H354" s="7" t="s">
@@ -13534,7 +13534,7 @@
       <c r="F355" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G355" s="55"/>
+      <c r="G355" s="60"/>
       <c r="H355" s="7" t="s">
         <v>420</v>
       </c>
@@ -13554,7 +13554,7 @@
       <c r="F356" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G356" s="55"/>
+      <c r="G356" s="60"/>
       <c r="H356" s="7" t="s">
         <v>420</v>
       </c>
@@ -13574,7 +13574,7 @@
       <c r="F357" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G357" s="55"/>
+      <c r="G357" s="60"/>
       <c r="H357" s="7" t="s">
         <v>420</v>
       </c>
@@ -13594,7 +13594,7 @@
       <c r="F358" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G358" s="55"/>
+      <c r="G358" s="60"/>
       <c r="H358" s="7" t="s">
         <v>420</v>
       </c>
@@ -13614,7 +13614,7 @@
       <c r="F359" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G359" s="55"/>
+      <c r="G359" s="60"/>
       <c r="H359" s="7" t="s">
         <v>420</v>
       </c>
@@ -35512,6 +35512,7 @@
     <hyperlink ref="C13:C19" r:id="rId3" display="aimy.tom@btech.christuniversity.in" xr:uid="{3F002A94-69C5-41DC-8EC0-9AC1A68C6030}"/>
     <hyperlink ref="C20" r:id="rId4" display="mailto:salomi.gopinath@btech.christuniversity.in" xr:uid="{D8C72E40-1E02-4D7D-BD92-5E424063D2B6}"/>
     <hyperlink ref="C21:C25" r:id="rId5" display="mailto:salomi.gopinath@btech.christuniversity.in" xr:uid="{7B5C7C44-96C2-4D84-94E3-E38F86C04500}"/>
+    <hyperlink ref="C3:C11" r:id="rId6" display="amaltomajithp@gmail.com" xr:uid="{4D01B2BF-770A-436E-B51D-7AF9D637D6BE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>